<commit_message>
Update 31 March report
</commit_message>
<xml_diff>
--- a/data/Mar/11-03-2026/NGAY 11-3.xlsx
+++ b/data/Mar/11-03-2026/NGAY 11-3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\TextExtractorTool\data\Mar\11-03-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Mar\11-03-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21505C34-0AD2-4515-B52A-A6DE85FFD916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BC73D1-1079-4798-96E3-D38C7EF50B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E69482-8B29-4E28-ACA9-4E97307A0D99}"/>
   </bookViews>
@@ -1245,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="J3" s="3">
-        <f>H3-I3</f>
+        <f t="shared" ref="J3:J25" si="0">H3-I3</f>
         <v>440</v>
       </c>
       <c r="K3" s="3" t="s">
@@ -1300,7 +1300,7 @@
         <v>0</v>
       </c>
       <c r="J4" s="3">
-        <f>H4-I4</f>
+        <f t="shared" si="0"/>
         <v>490</v>
       </c>
       <c r="K4" s="3" t="s">
@@ -1353,7 +1353,7 @@
         <v>25</v>
       </c>
       <c r="J5" s="2">
-        <f>H5-I5</f>
+        <f t="shared" si="0"/>
         <v>-25</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -1400,7 +1400,7 @@
         <v>30</v>
       </c>
       <c r="J6" s="35">
-        <f>H6-I6</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="K6" s="35" t="s">
@@ -1449,7 +1449,7 @@
         <v>25</v>
       </c>
       <c r="J7" s="2">
-        <f>H7-I7</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -1496,7 +1496,7 @@
         <v>20</v>
       </c>
       <c r="J8" s="2">
-        <f>H8-I8</f>
+        <f t="shared" si="0"/>
         <v>370</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -1543,7 +1543,7 @@
         <v>25</v>
       </c>
       <c r="J9" s="2">
-        <f>H9-I9</f>
+        <f t="shared" si="0"/>
         <v>370</v>
       </c>
       <c r="K9" s="2" t="s">
@@ -1590,7 +1590,7 @@
         <v>25</v>
       </c>
       <c r="J10" s="2">
-        <f>H10-I10</f>
+        <f t="shared" si="0"/>
         <v>580</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -1637,7 +1637,7 @@
         <v>25</v>
       </c>
       <c r="J11" s="2">
-        <f>H11-I11</f>
+        <f t="shared" si="0"/>
         <v>690</v>
       </c>
       <c r="K11" s="2" t="s">
@@ -1684,7 +1684,7 @@
         <v>20</v>
       </c>
       <c r="J12" s="2">
-        <f>H12-I12</f>
+        <f t="shared" si="0"/>
         <v>820</v>
       </c>
       <c r="K12" s="2" t="s">
@@ -1731,7 +1731,7 @@
         <v>30</v>
       </c>
       <c r="J13" s="2">
-        <f>H13-I13</f>
+        <f t="shared" si="0"/>
         <v>730</v>
       </c>
       <c r="K13" s="2" t="s">
@@ -1778,7 +1778,7 @@
         <v>25</v>
       </c>
       <c r="J14" s="2">
-        <f>H14-I14</f>
+        <f t="shared" si="0"/>
         <v>340</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -1825,7 +1825,7 @@
         <v>30</v>
       </c>
       <c r="J15" s="2">
-        <f>H15-I15</f>
+        <f t="shared" si="0"/>
         <v>-30</v>
       </c>
       <c r="K15" s="2" t="s">
@@ -1872,7 +1872,7 @@
         <v>30</v>
       </c>
       <c r="J16" s="2">
-        <f>H16-I16</f>
+        <f t="shared" si="0"/>
         <v>680</v>
       </c>
       <c r="K16" s="2" t="s">
@@ -1919,7 +1919,7 @@
         <v>50</v>
       </c>
       <c r="J17" s="2">
-        <f>H17-I17</f>
+        <f t="shared" si="0"/>
         <v>7800</v>
       </c>
       <c r="K17" s="2" t="s">
@@ -1966,7 +1966,7 @@
         <v>30</v>
       </c>
       <c r="J18" s="2">
-        <f>H18-I18</f>
+        <f t="shared" si="0"/>
         <v>1660</v>
       </c>
       <c r="K18" s="2" t="s">
@@ -2013,7 +2013,7 @@
         <v>30</v>
       </c>
       <c r="J19" s="35">
-        <f>H19-I19</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K19" s="35" t="s">
@@ -2062,7 +2062,7 @@
         <v>20</v>
       </c>
       <c r="J20" s="2">
-        <f>H20-I20</f>
+        <f t="shared" si="0"/>
         <v>-20</v>
       </c>
       <c r="K20" s="2" t="s">
@@ -2109,7 +2109,7 @@
         <v>20</v>
       </c>
       <c r="J21" s="2">
-        <f>H21-I21</f>
+        <f t="shared" si="0"/>
         <v>720</v>
       </c>
       <c r="K21" s="2" t="s">
@@ -2156,7 +2156,7 @@
         <v>25</v>
       </c>
       <c r="J22" s="2">
-        <f>H22-I22</f>
+        <f t="shared" si="0"/>
         <v>790</v>
       </c>
       <c r="K22" s="2" t="s">
@@ -2203,7 +2203,7 @@
         <v>25</v>
       </c>
       <c r="J23" s="2">
-        <f>H23-I23</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K23" s="2" t="s">
@@ -2250,7 +2250,7 @@
         <v>25</v>
       </c>
       <c r="J24" s="2">
-        <f>H24-I24</f>
+        <f t="shared" si="0"/>
         <v>1540</v>
       </c>
       <c r="K24" s="2" t="s">
@@ -2297,7 +2297,7 @@
         <v>30</v>
       </c>
       <c r="J25" s="2">
-        <f>H25-I25</f>
+        <f t="shared" si="0"/>
         <v>790</v>
       </c>
       <c r="K25" s="2" t="s">
@@ -2323,43 +2323,43 @@
         <v>20120</v>
       </c>
       <c r="I27">
-        <f t="shared" ref="I27:R27" si="0">SUBTOTAL(9,I3:I26)</f>
+        <f t="shared" ref="I27:R27" si="1">SUBTOTAL(9,I3:I26)</f>
         <v>565</v>
       </c>
       <c r="J27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>19555</v>
       </c>
       <c r="K27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="L27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="N27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="O27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="P27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Q27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
         <v>4600</v>
       </c>
       <c r="N35" s="31">
-        <f t="shared" ref="N35" si="1">SUBTOTAL(9,N30:N34)</f>
+        <f t="shared" ref="N35" si="2">SUBTOTAL(9,N30:N34)</f>
         <v>7</v>
       </c>
       <c r="P35" s="32" t="s">

</xml_diff>